<commit_message>
Update branding in Ops dataset README to Technizer India
</commit_message>
<xml_diff>
--- a/Ops_Copilot_Dataset.xlsx
+++ b/Ops_Copilot_Dataset.xlsx
@@ -2,7 +2,7 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
   <fileVersion appName="Calc"/>
-  <workbookPr backupFile="false" showObjects="all" date1904="false"/>
+  <workbookPr backupFile="false" showObjects="all" dateCompatibility="false"/>
   <workbookProtection/>
   <bookViews>
     <workbookView showHorizontalScroll="true" showVerticalScroll="true" showSheetTabs="true" xWindow="0" yWindow="0" windowWidth="16384" windowHeight="8192" tabRatio="500" firstSheet="0" activeTab="0"/>
@@ -27,7 +27,7 @@
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
 <sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="433" uniqueCount="310">
   <si>
-    <t xml:space="preserve">📖 Dataset Guide — Ops Team M365 Copilot Training | Technizer Edge</t>
+    <t xml:space="preserve">📖 Dataset Guide — Ops Team M365 Copilot Training | Technizer India</t>
   </si>
   <si>
     <t xml:space="preserve">Sheet</t>
@@ -1113,8 +1113,12 @@
     <xf numFmtId="42" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
     <xf numFmtId="9" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
   </cellStyleXfs>
-  <cellXfs count="9">
+  <cellXfs count="10">
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="false" applyProtection="false">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="true" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
@@ -1405,102 +1409,102 @@
   <dimension ref="A1:E7"/>
   <sheetFormatPr defaultColWidth="8.6796875" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="26"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="0" width="42"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="3" style="0" width="30"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="4" min="4" style="0" width="52"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="1" width="26"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="1" width="42"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="3" style="1" width="30"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="4" min="4" style="1" width="52"/>
   </cols>
   <sheetData>
     <row r="1" customFormat="false" ht="27.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A1" s="1" t="s">
-        <v>0</v>
-      </c>
-      <c r="B1" s="1"/>
-      <c r="C1" s="1"/>
-      <c r="D1" s="1"/>
-      <c r="E1" s="1"/>
+      <c r="A1" s="2" t="s">
+        <v>0</v>
+      </c>
+      <c r="B1" s="2"/>
+      <c r="C1" s="2"/>
+      <c r="D1" s="2"/>
+      <c r="E1" s="2"/>
     </row>
     <row r="2" customFormat="false" ht="36" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A2" s="2" t="s">
+      <c r="A2" s="3" t="s">
         <v>1</v>
       </c>
-      <c r="B2" s="2" t="s">
+      <c r="B2" s="3" t="s">
         <v>2</v>
       </c>
-      <c r="C2" s="2" t="s">
+      <c r="C2" s="3" t="s">
         <v>3</v>
       </c>
-      <c r="D2" s="2" t="s">
+      <c r="D2" s="3" t="s">
         <v>4</v>
       </c>
     </row>
-    <row r="3" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A3" s="3" t="s">
+    <row r="3" customFormat="false" ht="23.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A3" s="4" t="s">
         <v>5</v>
       </c>
-      <c r="B3" s="3" t="s">
+      <c r="B3" s="4" t="s">
         <v>6</v>
       </c>
-      <c r="C3" s="3" t="s">
+      <c r="C3" s="4" t="s">
         <v>7</v>
       </c>
-      <c r="D3" s="3" t="s">
+      <c r="D3" s="4" t="s">
         <v>8</v>
       </c>
     </row>
-    <row r="4" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A4" s="4" t="s">
+    <row r="4" customFormat="false" ht="23.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A4" s="5" t="s">
         <v>9</v>
       </c>
-      <c r="B4" s="4" t="s">
+      <c r="B4" s="5" t="s">
         <v>10</v>
       </c>
-      <c r="C4" s="4" t="s">
+      <c r="C4" s="5" t="s">
         <v>11</v>
       </c>
-      <c r="D4" s="4" t="s">
+      <c r="D4" s="5" t="s">
         <v>12</v>
       </c>
     </row>
-    <row r="5" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A5" s="5" t="s">
+    <row r="5" customFormat="false" ht="23.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A5" s="6" t="s">
         <v>13</v>
       </c>
-      <c r="B5" s="5" t="s">
+      <c r="B5" s="6" t="s">
         <v>14</v>
       </c>
-      <c r="C5" s="5" t="s">
+      <c r="C5" s="6" t="s">
         <v>15</v>
       </c>
-      <c r="D5" s="5" t="s">
+      <c r="D5" s="6" t="s">
         <v>16</v>
       </c>
     </row>
-    <row r="6" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A6" s="4" t="s">
+    <row r="6" customFormat="false" ht="23.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A6" s="5" t="s">
         <v>17</v>
       </c>
-      <c r="B6" s="4" t="s">
+      <c r="B6" s="5" t="s">
         <v>18</v>
       </c>
-      <c r="C6" s="4" t="s">
+      <c r="C6" s="5" t="s">
         <v>19</v>
       </c>
-      <c r="D6" s="4" t="s">
+      <c r="D6" s="5" t="s">
         <v>20</v>
       </c>
     </row>
-    <row r="7" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A7" s="5" t="s">
+    <row r="7" customFormat="false" ht="23.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A7" s="6" t="s">
         <v>21</v>
       </c>
-      <c r="B7" s="5" t="s">
+      <c r="B7" s="6" t="s">
         <v>22</v>
       </c>
-      <c r="C7" s="5" t="s">
+      <c r="C7" s="6" t="s">
         <v>23</v>
       </c>
-      <c r="D7" s="5" t="s">
+      <c r="D7" s="6" t="s">
         <v>24</v>
       </c>
     </row>
@@ -1526,403 +1530,403 @@
   <dimension ref="A1:I14"/>
   <sheetFormatPr defaultColWidth="8.6796875" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="14"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="0" width="34"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="3" style="0" width="18"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="4" min="4" style="0" width="16"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="5" min="5" style="0" width="10"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="6" min="6" style="0" width="14"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="7" min="7" style="0" width="12"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="9" min="8" style="0" width="14"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="1" width="14"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="1" width="34"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="3" style="1" width="18"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="4" min="4" style="1" width="16"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="5" min="5" style="1" width="10"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="6" min="6" style="1" width="14"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="7" min="7" style="1" width="12"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="9" min="8" style="1" width="14"/>
   </cols>
   <sheetData>
     <row r="1" customFormat="false" ht="27.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A1" s="1" t="s">
+      <c r="A1" s="2" t="s">
         <v>25</v>
       </c>
-      <c r="B1" s="1"/>
-      <c r="C1" s="1"/>
-      <c r="D1" s="1"/>
-      <c r="E1" s="1"/>
-      <c r="F1" s="1"/>
-      <c r="G1" s="1"/>
-      <c r="H1" s="1"/>
-      <c r="I1" s="1"/>
+      <c r="B1" s="2"/>
+      <c r="C1" s="2"/>
+      <c r="D1" s="2"/>
+      <c r="E1" s="2"/>
+      <c r="F1" s="2"/>
+      <c r="G1" s="2"/>
+      <c r="H1" s="2"/>
+      <c r="I1" s="2"/>
     </row>
     <row r="2" customFormat="false" ht="36" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A2" s="2" t="s">
+      <c r="A2" s="3" t="s">
         <v>26</v>
       </c>
-      <c r="B2" s="2" t="s">
+      <c r="B2" s="3" t="s">
         <v>27</v>
       </c>
-      <c r="C2" s="2" t="s">
+      <c r="C2" s="3" t="s">
         <v>28</v>
       </c>
-      <c r="D2" s="2" t="s">
+      <c r="D2" s="3" t="s">
         <v>29</v>
       </c>
-      <c r="E2" s="2" t="s">
+      <c r="E2" s="3" t="s">
         <v>30</v>
       </c>
-      <c r="F2" s="2" t="s">
+      <c r="F2" s="3" t="s">
         <v>31</v>
       </c>
-      <c r="G2" s="2" t="s">
+      <c r="G2" s="3" t="s">
         <v>32</v>
       </c>
-      <c r="H2" s="2" t="s">
+      <c r="H2" s="3" t="s">
         <v>33</v>
       </c>
-      <c r="I2" s="2" t="s">
+      <c r="I2" s="3" t="s">
         <v>34</v>
       </c>
     </row>
-    <row r="3" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A3" s="6" t="s">
+    <row r="3" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A3" s="7" t="s">
         <v>35</v>
       </c>
-      <c r="B3" s="6" t="s">
+      <c r="B3" s="7" t="s">
         <v>36</v>
       </c>
-      <c r="C3" s="6" t="s">
+      <c r="C3" s="7" t="s">
         <v>37</v>
       </c>
-      <c r="D3" s="6" t="s">
+      <c r="D3" s="7" t="s">
         <v>38</v>
       </c>
-      <c r="E3" s="6" t="s">
+      <c r="E3" s="7" t="s">
         <v>39</v>
       </c>
-      <c r="F3" s="6" t="s">
+      <c r="F3" s="7" t="s">
         <v>40</v>
       </c>
-      <c r="G3" s="6" t="s">
+      <c r="G3" s="7" t="s">
         <v>41</v>
       </c>
-      <c r="H3" s="6" t="s">
+      <c r="H3" s="7" t="s">
         <v>42</v>
       </c>
-      <c r="I3" s="6" t="s">
+      <c r="I3" s="7" t="s">
         <v>43</v>
       </c>
     </row>
-    <row r="4" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A4" s="7" t="s">
+    <row r="4" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A4" s="8" t="s">
         <v>44</v>
       </c>
-      <c r="B4" s="7" t="s">
+      <c r="B4" s="8" t="s">
         <v>45</v>
       </c>
-      <c r="C4" s="7" t="s">
+      <c r="C4" s="8" t="s">
         <v>46</v>
       </c>
-      <c r="D4" s="7" t="s">
+      <c r="D4" s="8" t="s">
         <v>47</v>
       </c>
-      <c r="E4" s="7" t="s">
+      <c r="E4" s="8" t="s">
         <v>48</v>
       </c>
-      <c r="F4" s="7" t="s">
+      <c r="F4" s="8" t="s">
         <v>49</v>
       </c>
-      <c r="G4" s="7" t="s">
+      <c r="G4" s="8" t="s">
         <v>50</v>
       </c>
-      <c r="H4" s="7" t="s">
+      <c r="H4" s="8" t="s">
         <v>42</v>
       </c>
-      <c r="I4" s="7" t="s">
+      <c r="I4" s="8" t="s">
         <v>43</v>
       </c>
     </row>
-    <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A5" s="6" t="s">
+    <row r="5" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A5" s="7" t="s">
         <v>51</v>
       </c>
-      <c r="B5" s="6" t="s">
+      <c r="B5" s="7" t="s">
         <v>52</v>
       </c>
-      <c r="C5" s="6" t="s">
+      <c r="C5" s="7" t="s">
         <v>53</v>
       </c>
-      <c r="D5" s="6" t="s">
+      <c r="D5" s="7" t="s">
         <v>54</v>
       </c>
-      <c r="E5" s="6" t="s">
+      <c r="E5" s="7" t="s">
         <v>55</v>
       </c>
-      <c r="F5" s="6" t="s">
+      <c r="F5" s="7" t="s">
         <v>56</v>
       </c>
-      <c r="G5" s="6" t="s">
+      <c r="G5" s="7" t="s">
         <v>57</v>
       </c>
-      <c r="H5" s="6" t="s">
+      <c r="H5" s="7" t="s">
         <v>58</v>
       </c>
-      <c r="I5" s="6" t="s">
+      <c r="I5" s="7" t="s">
         <v>43</v>
       </c>
     </row>
-    <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A6" s="7" t="s">
+    <row r="6" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A6" s="8" t="s">
         <v>59</v>
       </c>
-      <c r="B6" s="7" t="s">
+      <c r="B6" s="8" t="s">
         <v>60</v>
       </c>
-      <c r="C6" s="7" t="s">
+      <c r="C6" s="8" t="s">
         <v>61</v>
       </c>
-      <c r="D6" s="7" t="s">
+      <c r="D6" s="8" t="s">
         <v>62</v>
       </c>
-      <c r="E6" s="7" t="s">
+      <c r="E6" s="8" t="s">
         <v>63</v>
       </c>
-      <c r="F6" s="7" t="s">
+      <c r="F6" s="8" t="s">
         <v>64</v>
       </c>
-      <c r="G6" s="7" t="s">
+      <c r="G6" s="8" t="s">
         <v>65</v>
       </c>
-      <c r="H6" s="7" t="s">
+      <c r="H6" s="8" t="s">
         <v>42</v>
       </c>
-      <c r="I6" s="7" t="s">
+      <c r="I6" s="8" t="s">
         <v>66</v>
       </c>
     </row>
-    <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A7" s="6" t="s">
+    <row r="7" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A7" s="7" t="s">
         <v>67</v>
       </c>
-      <c r="B7" s="6" t="s">
+      <c r="B7" s="7" t="s">
         <v>68</v>
       </c>
-      <c r="C7" s="6" t="s">
+      <c r="C7" s="7" t="s">
         <v>69</v>
       </c>
-      <c r="D7" s="6" t="s">
+      <c r="D7" s="7" t="s">
         <v>70</v>
       </c>
-      <c r="E7" s="6" t="s">
+      <c r="E7" s="7" t="s">
         <v>71</v>
       </c>
-      <c r="F7" s="6" t="s">
+      <c r="F7" s="7" t="s">
         <v>72</v>
       </c>
-      <c r="G7" s="6" t="s">
+      <c r="G7" s="7" t="s">
         <v>73</v>
       </c>
-      <c r="H7" s="6" t="s">
+      <c r="H7" s="7" t="s">
         <v>74</v>
       </c>
-      <c r="I7" s="6" t="s">
+      <c r="I7" s="7" t="s">
         <v>66</v>
       </c>
     </row>
-    <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A8" s="7" t="s">
+    <row r="8" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A8" s="8" t="s">
         <v>75</v>
       </c>
-      <c r="B8" s="7" t="s">
+      <c r="B8" s="8" t="s">
         <v>76</v>
       </c>
-      <c r="C8" s="7" t="s">
+      <c r="C8" s="8" t="s">
         <v>77</v>
       </c>
-      <c r="D8" s="7" t="s">
+      <c r="D8" s="8" t="s">
         <v>78</v>
       </c>
-      <c r="E8" s="7" t="s">
+      <c r="E8" s="8" t="s">
         <v>79</v>
       </c>
-      <c r="F8" s="7" t="s">
+      <c r="F8" s="8" t="s">
         <v>40</v>
       </c>
-      <c r="G8" s="7" t="s">
+      <c r="G8" s="8" t="s">
         <v>41</v>
       </c>
-      <c r="H8" s="7" t="s">
+      <c r="H8" s="8" t="s">
         <v>42</v>
       </c>
-      <c r="I8" s="7" t="s">
+      <c r="I8" s="8" t="s">
         <v>43</v>
       </c>
     </row>
-    <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A9" s="6" t="s">
+    <row r="9" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A9" s="7" t="s">
         <v>80</v>
       </c>
-      <c r="B9" s="6" t="s">
+      <c r="B9" s="7" t="s">
         <v>81</v>
       </c>
-      <c r="C9" s="6" t="s">
+      <c r="C9" s="7" t="s">
         <v>82</v>
       </c>
-      <c r="D9" s="6" t="s">
+      <c r="D9" s="7" t="s">
         <v>83</v>
       </c>
-      <c r="E9" s="6" t="s">
+      <c r="E9" s="7" t="s">
         <v>84</v>
       </c>
-      <c r="F9" s="6" t="s">
+      <c r="F9" s="7" t="s">
         <v>49</v>
       </c>
-      <c r="G9" s="6" t="s">
+      <c r="G9" s="7" t="s">
         <v>50</v>
       </c>
-      <c r="H9" s="6" t="s">
+      <c r="H9" s="7" t="s">
         <v>42</v>
       </c>
-      <c r="I9" s="6" t="s">
+      <c r="I9" s="7" t="s">
         <v>43</v>
       </c>
     </row>
-    <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A10" s="7" t="s">
+    <row r="10" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A10" s="8" t="s">
         <v>85</v>
       </c>
-      <c r="B10" s="7" t="s">
+      <c r="B10" s="8" t="s">
         <v>86</v>
       </c>
-      <c r="C10" s="7" t="s">
+      <c r="C10" s="8" t="s">
         <v>87</v>
       </c>
-      <c r="D10" s="7" t="s">
+      <c r="D10" s="8" t="s">
         <v>88</v>
       </c>
-      <c r="E10" s="7" t="s">
+      <c r="E10" s="8" t="s">
         <v>89</v>
       </c>
-      <c r="F10" s="7" t="s">
+      <c r="F10" s="8" t="s">
         <v>90</v>
       </c>
-      <c r="G10" s="7" t="s">
+      <c r="G10" s="8" t="s">
         <v>91</v>
       </c>
-      <c r="H10" s="7" t="s">
+      <c r="H10" s="8" t="s">
         <v>74</v>
       </c>
-      <c r="I10" s="7" t="s">
+      <c r="I10" s="8" t="s">
         <v>92</v>
       </c>
     </row>
-    <row r="11" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A11" s="6" t="s">
+    <row r="11" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A11" s="7" t="s">
         <v>93</v>
       </c>
-      <c r="B11" s="6" t="s">
+      <c r="B11" s="7" t="s">
         <v>94</v>
       </c>
-      <c r="C11" s="6" t="s">
+      <c r="C11" s="7" t="s">
         <v>69</v>
       </c>
-      <c r="D11" s="6" t="s">
+      <c r="D11" s="7" t="s">
         <v>70</v>
       </c>
-      <c r="E11" s="6" t="s">
+      <c r="E11" s="7" t="s">
         <v>95</v>
       </c>
-      <c r="F11" s="6" t="s">
+      <c r="F11" s="7" t="s">
         <v>64</v>
       </c>
-      <c r="G11" s="6" t="s">
+      <c r="G11" s="7" t="s">
         <v>65</v>
       </c>
-      <c r="H11" s="6" t="s">
+      <c r="H11" s="7" t="s">
         <v>42</v>
       </c>
-      <c r="I11" s="6" t="s">
+      <c r="I11" s="7" t="s">
         <v>43</v>
       </c>
     </row>
-    <row r="12" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A12" s="7" t="s">
+    <row r="12" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A12" s="8" t="s">
         <v>96</v>
       </c>
-      <c r="B12" s="7" t="s">
+      <c r="B12" s="8" t="s">
         <v>97</v>
       </c>
-      <c r="C12" s="7" t="s">
+      <c r="C12" s="8" t="s">
         <v>98</v>
       </c>
-      <c r="D12" s="7" t="s">
+      <c r="D12" s="8" t="s">
         <v>99</v>
       </c>
-      <c r="E12" s="7" t="s">
+      <c r="E12" s="8" t="s">
         <v>100</v>
       </c>
-      <c r="F12" s="7" t="s">
+      <c r="F12" s="8" t="s">
         <v>40</v>
       </c>
-      <c r="G12" s="7" t="s">
+      <c r="G12" s="8" t="s">
         <v>41</v>
       </c>
-      <c r="H12" s="7" t="s">
+      <c r="H12" s="8" t="s">
         <v>42</v>
       </c>
-      <c r="I12" s="7" t="s">
+      <c r="I12" s="8" t="s">
         <v>101</v>
       </c>
     </row>
-    <row r="13" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A13" s="6" t="s">
+    <row r="13" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A13" s="7" t="s">
         <v>102</v>
       </c>
-      <c r="B13" s="6" t="s">
+      <c r="B13" s="7" t="s">
         <v>103</v>
       </c>
-      <c r="C13" s="6" t="s">
+      <c r="C13" s="7" t="s">
         <v>104</v>
       </c>
-      <c r="D13" s="6" t="s">
+      <c r="D13" s="7" t="s">
         <v>105</v>
       </c>
-      <c r="E13" s="6" t="s">
+      <c r="E13" s="7" t="s">
         <v>106</v>
       </c>
-      <c r="F13" s="6" t="s">
+      <c r="F13" s="7" t="s">
         <v>49</v>
       </c>
-      <c r="G13" s="6" t="s">
+      <c r="G13" s="7" t="s">
         <v>50</v>
       </c>
-      <c r="H13" s="6" t="s">
+      <c r="H13" s="7" t="s">
         <v>42</v>
       </c>
-      <c r="I13" s="6" t="s">
+      <c r="I13" s="7" t="s">
         <v>92</v>
       </c>
     </row>
-    <row r="14" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A14" s="7" t="s">
+    <row r="14" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A14" s="8" t="s">
         <v>107</v>
       </c>
-      <c r="B14" s="7" t="s">
+      <c r="B14" s="8" t="s">
         <v>108</v>
       </c>
-      <c r="C14" s="7" t="s">
+      <c r="C14" s="8" t="s">
         <v>98</v>
       </c>
-      <c r="D14" s="7" t="s">
+      <c r="D14" s="8" t="s">
         <v>99</v>
       </c>
-      <c r="E14" s="7" t="s">
+      <c r="E14" s="8" t="s">
         <v>109</v>
       </c>
-      <c r="F14" s="7" t="s">
+      <c r="F14" s="8" t="s">
         <v>64</v>
       </c>
-      <c r="G14" s="7" t="s">
+      <c r="G14" s="8" t="s">
         <v>65</v>
       </c>
-      <c r="H14" s="7" t="s">
+      <c r="H14" s="8" t="s">
         <v>42</v>
       </c>
-      <c r="I14" s="7" t="s">
+      <c r="I14" s="8" t="s">
         <v>101</v>
       </c>
     </row>
@@ -1948,483 +1952,483 @@
   <dimension ref="A1:K14"/>
   <sheetFormatPr defaultColWidth="8.6796875" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="1" style="0" width="14"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="3" style="0" width="22"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="4" min="4" style="0" width="10"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="5" min="5" style="0" width="22"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="6" min="6" style="0" width="46"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="7" min="7" style="0" width="14"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="10" min="8" style="0" width="18"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="11" min="11" style="0" width="12"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="1" style="1" width="14"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="3" style="1" width="22"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="4" min="4" style="1" width="10"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="5" min="5" style="1" width="22"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="6" min="6" style="1" width="46"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="7" min="7" style="1" width="14"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="10" min="8" style="1" width="18"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="11" min="11" style="1" width="12"/>
   </cols>
   <sheetData>
     <row r="1" customFormat="false" ht="27.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A1" s="1" t="s">
+      <c r="A1" s="2" t="s">
         <v>110</v>
       </c>
-      <c r="B1" s="1"/>
-      <c r="C1" s="1"/>
-      <c r="D1" s="1"/>
-      <c r="E1" s="1"/>
-      <c r="F1" s="1"/>
-      <c r="G1" s="1"/>
-      <c r="H1" s="1"/>
-      <c r="I1" s="1"/>
-      <c r="J1" s="1"/>
-      <c r="K1" s="1"/>
+      <c r="B1" s="2"/>
+      <c r="C1" s="2"/>
+      <c r="D1" s="2"/>
+      <c r="E1" s="2"/>
+      <c r="F1" s="2"/>
+      <c r="G1" s="2"/>
+      <c r="H1" s="2"/>
+      <c r="I1" s="2"/>
+      <c r="J1" s="2"/>
+      <c r="K1" s="2"/>
     </row>
     <row r="2" customFormat="false" ht="36" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A2" s="2" t="s">
+      <c r="A2" s="3" t="s">
         <v>111</v>
       </c>
-      <c r="B2" s="2" t="s">
+      <c r="B2" s="3" t="s">
         <v>112</v>
       </c>
-      <c r="C2" s="2" t="s">
+      <c r="C2" s="3" t="s">
         <v>113</v>
       </c>
-      <c r="D2" s="2" t="s">
+      <c r="D2" s="3" t="s">
         <v>114</v>
       </c>
-      <c r="E2" s="2" t="s">
+      <c r="E2" s="3" t="s">
         <v>115</v>
       </c>
-      <c r="F2" s="2" t="s">
+      <c r="F2" s="3" t="s">
         <v>116</v>
       </c>
-      <c r="G2" s="2" t="s">
+      <c r="G2" s="3" t="s">
         <v>117</v>
       </c>
-      <c r="H2" s="2" t="s">
+      <c r="H2" s="3" t="s">
         <v>118</v>
       </c>
-      <c r="I2" s="2" t="s">
+      <c r="I2" s="3" t="s">
         <v>119</v>
       </c>
-      <c r="J2" s="2" t="s">
+      <c r="J2" s="3" t="s">
         <v>33</v>
       </c>
-      <c r="K2" s="2" t="s">
+      <c r="K2" s="3" t="s">
         <v>120</v>
       </c>
     </row>
-    <row r="3" customFormat="false" ht="22.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A3" s="6" t="s">
+    <row r="3" customFormat="false" ht="21.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A3" s="7" t="s">
         <v>121</v>
       </c>
-      <c r="B3" s="6" t="s">
+      <c r="B3" s="7" t="s">
         <v>122</v>
       </c>
-      <c r="C3" s="6" t="s">
+      <c r="C3" s="7" t="s">
         <v>123</v>
       </c>
-      <c r="D3" s="6" t="s">
+      <c r="D3" s="7" t="s">
         <v>124</v>
       </c>
-      <c r="E3" s="6" t="s">
+      <c r="E3" s="7" t="s">
         <v>125</v>
       </c>
-      <c r="F3" s="6" t="s">
+      <c r="F3" s="7" t="s">
         <v>126</v>
       </c>
-      <c r="G3" s="6" t="n">
+      <c r="G3" s="7" t="n">
         <v>6</v>
       </c>
-      <c r="H3" s="6" t="n">
+      <c r="H3" s="7" t="n">
         <v>1240</v>
       </c>
-      <c r="I3" s="6" t="n">
+      <c r="I3" s="7" t="n">
         <v>9</v>
       </c>
-      <c r="J3" s="6" t="s">
+      <c r="J3" s="7" t="s">
         <v>127</v>
       </c>
-      <c r="K3" s="6" t="s">
+      <c r="K3" s="7" t="s">
         <v>128</v>
       </c>
     </row>
-    <row r="4" customFormat="false" ht="22.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A4" s="7" t="s">
+    <row r="4" customFormat="false" ht="21.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A4" s="8" t="s">
         <v>129</v>
       </c>
-      <c r="B4" s="7" t="s">
+      <c r="B4" s="8" t="s">
         <v>130</v>
       </c>
-      <c r="C4" s="7" t="s">
+      <c r="C4" s="8" t="s">
         <v>131</v>
       </c>
-      <c r="D4" s="7" t="s">
+      <c r="D4" s="8" t="s">
         <v>132</v>
       </c>
-      <c r="E4" s="7" t="s">
+      <c r="E4" s="8" t="s">
         <v>133</v>
       </c>
-      <c r="F4" s="7" t="s">
+      <c r="F4" s="8" t="s">
         <v>134</v>
       </c>
-      <c r="G4" s="7" t="n">
+      <c r="G4" s="8" t="n">
         <v>2</v>
       </c>
-      <c r="H4" s="7" t="n">
+      <c r="H4" s="8" t="n">
         <v>38</v>
       </c>
-      <c r="I4" s="7" t="n">
+      <c r="I4" s="8" t="n">
         <v>14</v>
       </c>
-      <c r="J4" s="7" t="s">
+      <c r="J4" s="8" t="s">
         <v>127</v>
       </c>
-      <c r="K4" s="7" t="s">
+      <c r="K4" s="8" t="s">
         <v>135</v>
       </c>
     </row>
-    <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A5" s="6" t="s">
+    <row r="5" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A5" s="7" t="s">
         <v>136</v>
       </c>
-      <c r="B5" s="6" t="s">
+      <c r="B5" s="7" t="s">
         <v>137</v>
       </c>
-      <c r="C5" s="6" t="s">
+      <c r="C5" s="7" t="s">
         <v>138</v>
       </c>
-      <c r="D5" s="6" t="s">
+      <c r="D5" s="7" t="s">
         <v>132</v>
       </c>
-      <c r="E5" s="6" t="s">
+      <c r="E5" s="7" t="s">
         <v>139</v>
       </c>
-      <c r="F5" s="6" t="s">
+      <c r="F5" s="7" t="s">
         <v>140</v>
       </c>
-      <c r="G5" s="6" t="n">
+      <c r="G5" s="7" t="n">
         <v>3</v>
       </c>
-      <c r="H5" s="6" t="n">
+      <c r="H5" s="7" t="n">
         <v>520</v>
       </c>
-      <c r="I5" s="6" t="n">
+      <c r="I5" s="7" t="n">
         <v>6</v>
       </c>
-      <c r="J5" s="6" t="s">
+      <c r="J5" s="7" t="s">
         <v>127</v>
       </c>
-      <c r="K5" s="6" t="s">
+      <c r="K5" s="7" t="s">
         <v>128</v>
       </c>
     </row>
-    <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A6" s="7" t="s">
+    <row r="6" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A6" s="8" t="s">
         <v>141</v>
       </c>
-      <c r="B6" s="7" t="s">
+      <c r="B6" s="8" t="s">
         <v>142</v>
       </c>
-      <c r="C6" s="7" t="s">
+      <c r="C6" s="8" t="s">
         <v>143</v>
       </c>
-      <c r="D6" s="7" t="s">
+      <c r="D6" s="8" t="s">
         <v>124</v>
       </c>
-      <c r="E6" s="7" t="s">
+      <c r="E6" s="8" t="s">
         <v>144</v>
       </c>
-      <c r="F6" s="7" t="s">
+      <c r="F6" s="8" t="s">
         <v>145</v>
       </c>
-      <c r="G6" s="7" t="n">
-        <v>0</v>
-      </c>
-      <c r="H6" s="7" t="n">
-        <v>0</v>
-      </c>
-      <c r="I6" s="7" t="n">
+      <c r="G6" s="8" t="n">
+        <v>0</v>
+      </c>
+      <c r="H6" s="8" t="n">
+        <v>0</v>
+      </c>
+      <c r="I6" s="8" t="n">
         <v>18</v>
       </c>
-      <c r="J6" s="7" t="s">
+      <c r="J6" s="8" t="s">
         <v>127</v>
       </c>
-      <c r="K6" s="7" t="s">
+      <c r="K6" s="8" t="s">
         <v>128</v>
       </c>
     </row>
-    <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A7" s="6" t="s">
+    <row r="7" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A7" s="7" t="s">
         <v>146</v>
       </c>
-      <c r="B7" s="6" t="s">
+      <c r="B7" s="7" t="s">
         <v>147</v>
       </c>
-      <c r="C7" s="6" t="s">
+      <c r="C7" s="7" t="s">
         <v>148</v>
       </c>
-      <c r="D7" s="6" t="s">
+      <c r="D7" s="7" t="s">
         <v>132</v>
       </c>
-      <c r="E7" s="6" t="s">
+      <c r="E7" s="7" t="s">
         <v>133</v>
       </c>
-      <c r="F7" s="6" t="s">
+      <c r="F7" s="7" t="s">
         <v>149</v>
       </c>
-      <c r="G7" s="6" t="n">
-        <v>0</v>
-      </c>
-      <c r="H7" s="6" t="n">
-        <v>0</v>
-      </c>
-      <c r="I7" s="6" t="n">
+      <c r="G7" s="7" t="n">
+        <v>0</v>
+      </c>
+      <c r="H7" s="7" t="n">
+        <v>0</v>
+      </c>
+      <c r="I7" s="7" t="n">
         <v>36</v>
       </c>
-      <c r="J7" s="6" t="s">
+      <c r="J7" s="7" t="s">
         <v>127</v>
       </c>
-      <c r="K7" s="6" t="s">
+      <c r="K7" s="7" t="s">
         <v>135</v>
       </c>
     </row>
-    <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A8" s="7" t="s">
+    <row r="8" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A8" s="8" t="s">
         <v>150</v>
       </c>
-      <c r="B8" s="7" t="s">
+      <c r="B8" s="8" t="s">
         <v>151</v>
       </c>
-      <c r="C8" s="7" t="s">
+      <c r="C8" s="8" t="s">
         <v>152</v>
       </c>
-      <c r="D8" s="7" t="s">
+      <c r="D8" s="8" t="s">
         <v>153</v>
       </c>
-      <c r="E8" s="7" t="s">
+      <c r="E8" s="8" t="s">
         <v>154</v>
       </c>
-      <c r="F8" s="7" t="s">
+      <c r="F8" s="8" t="s">
         <v>155</v>
       </c>
-      <c r="G8" s="7" t="n">
+      <c r="G8" s="8" t="n">
         <v>1</v>
       </c>
-      <c r="H8" s="7" t="n">
+      <c r="H8" s="8" t="n">
         <v>12</v>
       </c>
-      <c r="I8" s="7" t="n">
+      <c r="I8" s="8" t="n">
         <v>8</v>
       </c>
-      <c r="J8" s="7" t="s">
+      <c r="J8" s="8" t="s">
         <v>127</v>
       </c>
-      <c r="K8" s="7" t="s">
+      <c r="K8" s="8" t="s">
         <v>135</v>
       </c>
     </row>
-    <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A9" s="6" t="s">
+    <row r="9" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A9" s="7" t="s">
         <v>156</v>
       </c>
-      <c r="B9" s="6" t="s">
+      <c r="B9" s="7" t="s">
         <v>157</v>
       </c>
-      <c r="C9" s="6" t="s">
+      <c r="C9" s="7" t="s">
         <v>158</v>
       </c>
-      <c r="D9" s="6" t="s">
+      <c r="D9" s="7" t="s">
         <v>132</v>
       </c>
-      <c r="E9" s="6" t="s">
+      <c r="E9" s="7" t="s">
         <v>125</v>
       </c>
-      <c r="F9" s="6" t="s">
+      <c r="F9" s="7" t="s">
         <v>159</v>
       </c>
-      <c r="G9" s="6" t="n">
-        <v>0</v>
-      </c>
-      <c r="H9" s="6" t="n">
-        <v>0</v>
-      </c>
-      <c r="I9" s="6" t="n">
+      <c r="G9" s="7" t="n">
+        <v>0</v>
+      </c>
+      <c r="H9" s="7" t="n">
+        <v>0</v>
+      </c>
+      <c r="I9" s="7" t="n">
         <v>24</v>
       </c>
-      <c r="J9" s="6" t="s">
+      <c r="J9" s="7" t="s">
         <v>127</v>
       </c>
-      <c r="K9" s="6" t="s">
+      <c r="K9" s="7" t="s">
         <v>128</v>
       </c>
     </row>
-    <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A10" s="7" t="s">
+    <row r="10" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A10" s="8" t="s">
         <v>160</v>
       </c>
-      <c r="B10" s="7" t="s">
+      <c r="B10" s="8" t="s">
         <v>161</v>
       </c>
-      <c r="C10" s="7" t="s">
+      <c r="C10" s="8" t="s">
         <v>162</v>
       </c>
-      <c r="D10" s="7" t="s">
+      <c r="D10" s="8" t="s">
         <v>153</v>
       </c>
-      <c r="E10" s="7" t="s">
+      <c r="E10" s="8" t="s">
         <v>154</v>
       </c>
-      <c r="F10" s="7" t="s">
+      <c r="F10" s="8" t="s">
         <v>163</v>
       </c>
-      <c r="G10" s="7" t="n">
-        <v>0</v>
-      </c>
-      <c r="H10" s="7" t="n">
+      <c r="G10" s="8" t="n">
+        <v>0</v>
+      </c>
+      <c r="H10" s="8" t="n">
         <v>1</v>
       </c>
-      <c r="I10" s="7" t="n">
+      <c r="I10" s="8" t="n">
         <v>4</v>
       </c>
-      <c r="J10" s="7" t="s">
+      <c r="J10" s="8" t="s">
         <v>127</v>
       </c>
-      <c r="K10" s="7" t="s">
+      <c r="K10" s="8" t="s">
         <v>128</v>
       </c>
     </row>
-    <row r="11" customFormat="false" ht="22.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A11" s="6" t="s">
+    <row r="11" customFormat="false" ht="21.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A11" s="7" t="s">
         <v>164</v>
       </c>
-      <c r="B11" s="6" t="s">
+      <c r="B11" s="7" t="s">
         <v>165</v>
       </c>
-      <c r="C11" s="6" t="s">
+      <c r="C11" s="7" t="s">
         <v>166</v>
       </c>
-      <c r="D11" s="6" t="s">
+      <c r="D11" s="7" t="s">
         <v>153</v>
       </c>
-      <c r="E11" s="6" t="s">
+      <c r="E11" s="7" t="s">
         <v>133</v>
       </c>
-      <c r="F11" s="6" t="s">
+      <c r="F11" s="7" t="s">
         <v>167</v>
       </c>
-      <c r="G11" s="6" t="n">
-        <v>0</v>
-      </c>
-      <c r="H11" s="6" t="n">
-        <v>0</v>
-      </c>
-      <c r="I11" s="6" t="n">
+      <c r="G11" s="7" t="n">
+        <v>0</v>
+      </c>
+      <c r="H11" s="7" t="n">
+        <v>0</v>
+      </c>
+      <c r="I11" s="7" t="n">
         <v>12</v>
       </c>
-      <c r="J11" s="6" t="s">
+      <c r="J11" s="7" t="s">
         <v>168</v>
       </c>
-      <c r="K11" s="6" t="s">
+      <c r="K11" s="7" t="s">
         <v>128</v>
       </c>
     </row>
-    <row r="12" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A12" s="7" t="s">
+    <row r="12" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A12" s="8" t="s">
         <v>169</v>
       </c>
-      <c r="B12" s="7" t="s">
+      <c r="B12" s="8" t="s">
         <v>170</v>
       </c>
-      <c r="C12" s="7" t="s">
+      <c r="C12" s="8" t="s">
         <v>123</v>
       </c>
-      <c r="D12" s="7" t="s">
+      <c r="D12" s="8" t="s">
         <v>132</v>
       </c>
-      <c r="E12" s="7" t="s">
+      <c r="E12" s="8" t="s">
         <v>139</v>
       </c>
-      <c r="F12" s="7" t="s">
+      <c r="F12" s="8" t="s">
         <v>171</v>
       </c>
-      <c r="G12" s="7" t="n">
+      <c r="G12" s="8" t="n">
         <v>3</v>
       </c>
-      <c r="H12" s="7" t="n">
+      <c r="H12" s="8" t="n">
         <v>680</v>
       </c>
-      <c r="I12" s="7" t="n">
+      <c r="I12" s="8" t="n">
         <v>5</v>
       </c>
-      <c r="J12" s="7" t="s">
+      <c r="J12" s="8" t="s">
         <v>127</v>
       </c>
-      <c r="K12" s="7" t="s">
+      <c r="K12" s="8" t="s">
         <v>135</v>
       </c>
     </row>
-    <row r="13" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A13" s="6" t="s">
+    <row r="13" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A13" s="7" t="s">
         <v>172</v>
       </c>
-      <c r="B13" s="6" t="s">
+      <c r="B13" s="7" t="s">
         <v>173</v>
       </c>
-      <c r="C13" s="6" t="s">
+      <c r="C13" s="7" t="s">
         <v>174</v>
       </c>
-      <c r="D13" s="6" t="s">
+      <c r="D13" s="7" t="s">
         <v>132</v>
       </c>
-      <c r="E13" s="6" t="s">
+      <c r="E13" s="7" t="s">
         <v>144</v>
       </c>
-      <c r="F13" s="6" t="s">
+      <c r="F13" s="7" t="s">
         <v>175</v>
       </c>
-      <c r="G13" s="6" t="n">
+      <c r="G13" s="7" t="n">
         <v>2</v>
       </c>
-      <c r="H13" s="6" t="n">
+      <c r="H13" s="7" t="n">
         <v>290</v>
       </c>
-      <c r="I13" s="6" t="n">
+      <c r="I13" s="7" t="n">
         <v>7</v>
       </c>
-      <c r="J13" s="6" t="s">
+      <c r="J13" s="7" t="s">
         <v>176</v>
       </c>
-      <c r="K13" s="6" t="s">
+      <c r="K13" s="7" t="s">
         <v>128</v>
       </c>
     </row>
-    <row r="14" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A14" s="7" t="s">
+    <row r="14" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A14" s="8" t="s">
         <v>177</v>
       </c>
-      <c r="B14" s="7" t="s">
+      <c r="B14" s="8" t="s">
         <v>173</v>
       </c>
-      <c r="C14" s="7" t="s">
+      <c r="C14" s="8" t="s">
         <v>148</v>
       </c>
-      <c r="D14" s="7" t="s">
+      <c r="D14" s="8" t="s">
         <v>124</v>
       </c>
-      <c r="E14" s="7" t="s">
+      <c r="E14" s="8" t="s">
         <v>178</v>
       </c>
-      <c r="F14" s="7" t="s">
+      <c r="F14" s="8" t="s">
         <v>179</v>
       </c>
-      <c r="G14" s="7" t="n">
-        <v>0</v>
-      </c>
-      <c r="H14" s="7" t="n">
-        <v>0</v>
-      </c>
-      <c r="I14" s="7" t="n">
-        <v>0</v>
-      </c>
-      <c r="J14" s="7" t="s">
+      <c r="G14" s="8" t="n">
+        <v>0</v>
+      </c>
+      <c r="H14" s="8" t="n">
+        <v>0</v>
+      </c>
+      <c r="I14" s="8" t="n">
+        <v>0</v>
+      </c>
+      <c r="J14" s="8" t="s">
         <v>180</v>
       </c>
-      <c r="K14" s="7" t="s">
+      <c r="K14" s="8" t="s">
         <v>128</v>
       </c>
     </row>
@@ -2450,484 +2454,484 @@
   <dimension ref="A1:J15"/>
   <sheetFormatPr defaultColWidth="8.6796875" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="14"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="0" width="22"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="4" min="3" style="0" width="18"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="5" min="5" style="0" width="22"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="6" min="6" style="0" width="14"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="7" min="7" style="0" width="22"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="8" min="8" style="0" width="20"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="9" min="9" style="0" width="14"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="10" min="10" style="0" width="18"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="1" width="14"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="1" width="22"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="4" min="3" style="1" width="18"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="5" min="5" style="1" width="22"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="6" min="6" style="1" width="14"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="7" min="7" style="1" width="22"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="8" min="8" style="1" width="20"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="9" min="9" style="1" width="14"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="10" min="10" style="1" width="18"/>
   </cols>
   <sheetData>
     <row r="1" customFormat="false" ht="27.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A1" s="1" t="s">
+      <c r="A1" s="2" t="s">
         <v>181</v>
       </c>
-      <c r="B1" s="1"/>
-      <c r="C1" s="1"/>
-      <c r="D1" s="1"/>
-      <c r="E1" s="1"/>
-      <c r="F1" s="1"/>
-      <c r="G1" s="1"/>
-      <c r="H1" s="1"/>
-      <c r="I1" s="1"/>
-      <c r="J1" s="1"/>
+      <c r="B1" s="2"/>
+      <c r="C1" s="2"/>
+      <c r="D1" s="2"/>
+      <c r="E1" s="2"/>
+      <c r="F1" s="2"/>
+      <c r="G1" s="2"/>
+      <c r="H1" s="2"/>
+      <c r="I1" s="2"/>
+      <c r="J1" s="2"/>
     </row>
     <row r="2" customFormat="false" ht="36" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A2" s="2" t="s">
+      <c r="A2" s="3" t="s">
         <v>182</v>
       </c>
-      <c r="B2" s="2" t="s">
+      <c r="B2" s="3" t="s">
         <v>183</v>
       </c>
-      <c r="C2" s="2" t="s">
+      <c r="C2" s="3" t="s">
         <v>184</v>
       </c>
-      <c r="D2" s="2" t="s">
+      <c r="D2" s="3" t="s">
         <v>185</v>
       </c>
-      <c r="E2" s="2" t="s">
+      <c r="E2" s="3" t="s">
         <v>186</v>
       </c>
-      <c r="F2" s="2" t="s">
+      <c r="F2" s="3" t="s">
         <v>187</v>
       </c>
-      <c r="G2" s="2" t="s">
+      <c r="G2" s="3" t="s">
         <v>188</v>
       </c>
-      <c r="H2" s="2" t="s">
+      <c r="H2" s="3" t="s">
         <v>189</v>
       </c>
-      <c r="I2" s="2" t="s">
+      <c r="I2" s="3" t="s">
         <v>190</v>
       </c>
-      <c r="J2" s="2" t="s">
+      <c r="J2" s="3" t="s">
         <v>191</v>
       </c>
     </row>
-    <row r="3" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A3" s="6" t="s">
+    <row r="3" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A3" s="7" t="s">
         <v>91</v>
       </c>
-      <c r="B3" s="6" t="n">
+      <c r="B3" s="7" t="n">
         <v>142800</v>
       </c>
-      <c r="C3" s="6" t="n">
+      <c r="C3" s="7" t="n">
         <v>94.2</v>
       </c>
-      <c r="D3" s="6" t="n">
+      <c r="D3" s="7" t="n">
         <v>88.6</v>
       </c>
-      <c r="E3" s="6" t="n">
+      <c r="E3" s="7" t="n">
         <v>1.8</v>
       </c>
-      <c r="F3" s="6" t="n">
+      <c r="F3" s="7" t="n">
         <v>1.4</v>
       </c>
-      <c r="G3" s="6" t="n">
+      <c r="G3" s="7" t="n">
         <v>48.2</v>
       </c>
-      <c r="H3" s="6" t="n">
+      <c r="H3" s="7" t="n">
         <v>312</v>
       </c>
-      <c r="I3" s="6" t="n">
+      <c r="I3" s="7" t="n">
         <v>28</v>
       </c>
-      <c r="J3" s="6" t="n">
+      <c r="J3" s="7" t="n">
         <v>3</v>
       </c>
     </row>
-    <row r="4" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A4" s="7" t="s">
+    <row r="4" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A4" s="8" t="s">
         <v>73</v>
       </c>
-      <c r="B4" s="7" t="n">
+      <c r="B4" s="8" t="n">
         <v>138500</v>
       </c>
-      <c r="C4" s="7" t="n">
+      <c r="C4" s="8" t="n">
         <v>93.8</v>
       </c>
-      <c r="D4" s="7" t="n">
+      <c r="D4" s="8" t="n">
         <v>89.1</v>
       </c>
-      <c r="E4" s="7" t="n">
+      <c r="E4" s="8" t="n">
         <v>1.9</v>
       </c>
-      <c r="F4" s="7" t="n">
+      <c r="F4" s="8" t="n">
         <v>1.6</v>
       </c>
-      <c r="G4" s="7" t="n">
+      <c r="G4" s="8" t="n">
         <v>49.1</v>
       </c>
-      <c r="H4" s="7" t="n">
+      <c r="H4" s="8" t="n">
         <v>298</v>
       </c>
-      <c r="I4" s="7" t="n">
+      <c r="I4" s="8" t="n">
         <v>31</v>
       </c>
-      <c r="J4" s="7" t="n">
+      <c r="J4" s="8" t="n">
         <v>4</v>
       </c>
     </row>
-    <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A5" s="6" t="s">
+    <row r="5" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A5" s="7" t="s">
         <v>57</v>
       </c>
-      <c r="B5" s="6" t="n">
+      <c r="B5" s="7" t="n">
         <v>145200</v>
       </c>
-      <c r="C5" s="6" t="n">
+      <c r="C5" s="7" t="n">
         <v>91.5</v>
       </c>
-      <c r="D5" s="6" t="n">
+      <c r="D5" s="7" t="n">
         <v>87.4</v>
       </c>
-      <c r="E5" s="6" t="n">
+      <c r="E5" s="7" t="n">
         <v>2.1</v>
       </c>
-      <c r="F5" s="6" t="n">
+      <c r="F5" s="7" t="n">
         <v>2.2</v>
       </c>
-      <c r="G5" s="6" t="n">
+      <c r="G5" s="7" t="n">
         <v>51.4</v>
       </c>
-      <c r="H5" s="6" t="n">
+      <c r="H5" s="7" t="n">
         <v>386</v>
       </c>
-      <c r="I5" s="6" t="n">
+      <c r="I5" s="7" t="n">
         <v>45</v>
       </c>
-      <c r="J5" s="6" t="n">
+      <c r="J5" s="7" t="n">
         <v>3</v>
       </c>
     </row>
-    <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A6" s="7" t="s">
+    <row r="6" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A6" s="8" t="s">
         <v>41</v>
       </c>
-      <c r="B6" s="7" t="n">
-        <v>0</v>
-      </c>
-      <c r="C6" s="7" t="n">
-        <v>0</v>
-      </c>
-      <c r="D6" s="7" t="n">
-        <v>0</v>
-      </c>
-      <c r="E6" s="7" t="n">
-        <v>0</v>
-      </c>
-      <c r="F6" s="7" t="n">
-        <v>0</v>
-      </c>
-      <c r="G6" s="7" t="n">
-        <v>0</v>
-      </c>
-      <c r="H6" s="7" t="n">
-        <v>0</v>
-      </c>
-      <c r="I6" s="7" t="n">
-        <v>0</v>
-      </c>
-      <c r="J6" s="7" t="n">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A7" s="6" t="s">
+      <c r="B6" s="8" t="n">
+        <v>0</v>
+      </c>
+      <c r="C6" s="8" t="n">
+        <v>0</v>
+      </c>
+      <c r="D6" s="8" t="n">
+        <v>0</v>
+      </c>
+      <c r="E6" s="8" t="n">
+        <v>0</v>
+      </c>
+      <c r="F6" s="8" t="n">
+        <v>0</v>
+      </c>
+      <c r="G6" s="8" t="n">
+        <v>0</v>
+      </c>
+      <c r="H6" s="8" t="n">
+        <v>0</v>
+      </c>
+      <c r="I6" s="8" t="n">
+        <v>0</v>
+      </c>
+      <c r="J6" s="8" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="7" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A7" s="7" t="s">
         <v>50</v>
       </c>
-      <c r="B7" s="6" t="n">
-        <v>0</v>
-      </c>
-      <c r="C7" s="6" t="n">
-        <v>0</v>
-      </c>
-      <c r="D7" s="6" t="n">
-        <v>0</v>
-      </c>
-      <c r="E7" s="6" t="n">
-        <v>0</v>
-      </c>
-      <c r="F7" s="6" t="n">
-        <v>0</v>
-      </c>
-      <c r="G7" s="6" t="n">
-        <v>0</v>
-      </c>
-      <c r="H7" s="6" t="n">
-        <v>0</v>
-      </c>
-      <c r="I7" s="6" t="n">
-        <v>0</v>
-      </c>
-      <c r="J7" s="6" t="n">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A8" s="7" t="s">
+      <c r="B7" s="7" t="n">
+        <v>0</v>
+      </c>
+      <c r="C7" s="7" t="n">
+        <v>0</v>
+      </c>
+      <c r="D7" s="7" t="n">
+        <v>0</v>
+      </c>
+      <c r="E7" s="7" t="n">
+        <v>0</v>
+      </c>
+      <c r="F7" s="7" t="n">
+        <v>0</v>
+      </c>
+      <c r="G7" s="7" t="n">
+        <v>0</v>
+      </c>
+      <c r="H7" s="7" t="n">
+        <v>0</v>
+      </c>
+      <c r="I7" s="7" t="n">
+        <v>0</v>
+      </c>
+      <c r="J7" s="7" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="8" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A8" s="8" t="s">
         <v>65</v>
       </c>
-      <c r="B8" s="7" t="n">
-        <v>0</v>
-      </c>
-      <c r="C8" s="7" t="n">
-        <v>0</v>
-      </c>
-      <c r="D8" s="7" t="n">
-        <v>0</v>
-      </c>
-      <c r="E8" s="7" t="n">
-        <v>0</v>
-      </c>
-      <c r="F8" s="7" t="n">
-        <v>0</v>
-      </c>
-      <c r="G8" s="7" t="n">
-        <v>0</v>
-      </c>
-      <c r="H8" s="7" t="n">
-        <v>0</v>
-      </c>
-      <c r="I8" s="7" t="n">
-        <v>0</v>
-      </c>
-      <c r="J8" s="7" t="n">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A9" s="6" t="s">
+      <c r="B8" s="8" t="n">
+        <v>0</v>
+      </c>
+      <c r="C8" s="8" t="n">
+        <v>0</v>
+      </c>
+      <c r="D8" s="8" t="n">
+        <v>0</v>
+      </c>
+      <c r="E8" s="8" t="n">
+        <v>0</v>
+      </c>
+      <c r="F8" s="8" t="n">
+        <v>0</v>
+      </c>
+      <c r="G8" s="8" t="n">
+        <v>0</v>
+      </c>
+      <c r="H8" s="8" t="n">
+        <v>0</v>
+      </c>
+      <c r="I8" s="8" t="n">
+        <v>0</v>
+      </c>
+      <c r="J8" s="8" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="9" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A9" s="7" t="s">
         <v>192</v>
       </c>
-      <c r="B9" s="6" t="n">
-        <v>0</v>
-      </c>
-      <c r="C9" s="6" t="n">
-        <v>0</v>
-      </c>
-      <c r="D9" s="6" t="n">
-        <v>0</v>
-      </c>
-      <c r="E9" s="6" t="n">
-        <v>0</v>
-      </c>
-      <c r="F9" s="6" t="n">
-        <v>0</v>
-      </c>
-      <c r="G9" s="6" t="n">
-        <v>0</v>
-      </c>
-      <c r="H9" s="6" t="n">
-        <v>0</v>
-      </c>
-      <c r="I9" s="6" t="n">
-        <v>0</v>
-      </c>
-      <c r="J9" s="6" t="n">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A10" s="7" t="s">
+      <c r="B9" s="7" t="n">
+        <v>0</v>
+      </c>
+      <c r="C9" s="7" t="n">
+        <v>0</v>
+      </c>
+      <c r="D9" s="7" t="n">
+        <v>0</v>
+      </c>
+      <c r="E9" s="7" t="n">
+        <v>0</v>
+      </c>
+      <c r="F9" s="7" t="n">
+        <v>0</v>
+      </c>
+      <c r="G9" s="7" t="n">
+        <v>0</v>
+      </c>
+      <c r="H9" s="7" t="n">
+        <v>0</v>
+      </c>
+      <c r="I9" s="7" t="n">
+        <v>0</v>
+      </c>
+      <c r="J9" s="7" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="10" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A10" s="8" t="s">
         <v>193</v>
       </c>
-      <c r="B10" s="7" t="n">
-        <v>0</v>
-      </c>
-      <c r="C10" s="7" t="n">
-        <v>0</v>
-      </c>
-      <c r="D10" s="7" t="n">
-        <v>0</v>
-      </c>
-      <c r="E10" s="7" t="n">
-        <v>0</v>
-      </c>
-      <c r="F10" s="7" t="n">
-        <v>0</v>
-      </c>
-      <c r="G10" s="7" t="n">
-        <v>0</v>
-      </c>
-      <c r="H10" s="7" t="n">
-        <v>0</v>
-      </c>
-      <c r="I10" s="7" t="n">
-        <v>0</v>
-      </c>
-      <c r="J10" s="7" t="n">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="11" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A11" s="6" t="s">
+      <c r="B10" s="8" t="n">
+        <v>0</v>
+      </c>
+      <c r="C10" s="8" t="n">
+        <v>0</v>
+      </c>
+      <c r="D10" s="8" t="n">
+        <v>0</v>
+      </c>
+      <c r="E10" s="8" t="n">
+        <v>0</v>
+      </c>
+      <c r="F10" s="8" t="n">
+        <v>0</v>
+      </c>
+      <c r="G10" s="8" t="n">
+        <v>0</v>
+      </c>
+      <c r="H10" s="8" t="n">
+        <v>0</v>
+      </c>
+      <c r="I10" s="8" t="n">
+        <v>0</v>
+      </c>
+      <c r="J10" s="8" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="11" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A11" s="7" t="s">
         <v>194</v>
       </c>
-      <c r="B11" s="6" t="n">
-        <v>0</v>
-      </c>
-      <c r="C11" s="6" t="n">
-        <v>0</v>
-      </c>
-      <c r="D11" s="6" t="n">
-        <v>0</v>
-      </c>
-      <c r="E11" s="6" t="n">
-        <v>0</v>
-      </c>
-      <c r="F11" s="6" t="n">
-        <v>0</v>
-      </c>
-      <c r="G11" s="6" t="n">
-        <v>0</v>
-      </c>
-      <c r="H11" s="6" t="n">
-        <v>0</v>
-      </c>
-      <c r="I11" s="6" t="n">
-        <v>0</v>
-      </c>
-      <c r="J11" s="6" t="n">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="12" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A12" s="7" t="s">
+      <c r="B11" s="7" t="n">
+        <v>0</v>
+      </c>
+      <c r="C11" s="7" t="n">
+        <v>0</v>
+      </c>
+      <c r="D11" s="7" t="n">
+        <v>0</v>
+      </c>
+      <c r="E11" s="7" t="n">
+        <v>0</v>
+      </c>
+      <c r="F11" s="7" t="n">
+        <v>0</v>
+      </c>
+      <c r="G11" s="7" t="n">
+        <v>0</v>
+      </c>
+      <c r="H11" s="7" t="n">
+        <v>0</v>
+      </c>
+      <c r="I11" s="7" t="n">
+        <v>0</v>
+      </c>
+      <c r="J11" s="7" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="12" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A12" s="8" t="s">
         <v>195</v>
       </c>
-      <c r="B12" s="7" t="n">
-        <v>0</v>
-      </c>
-      <c r="C12" s="7" t="n">
-        <v>0</v>
-      </c>
-      <c r="D12" s="7" t="n">
-        <v>0</v>
-      </c>
-      <c r="E12" s="7" t="n">
-        <v>0</v>
-      </c>
-      <c r="F12" s="7" t="n">
-        <v>0</v>
-      </c>
-      <c r="G12" s="7" t="n">
-        <v>0</v>
-      </c>
-      <c r="H12" s="7" t="n">
-        <v>0</v>
-      </c>
-      <c r="I12" s="7" t="n">
-        <v>0</v>
-      </c>
-      <c r="J12" s="7" t="n">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="13" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A13" s="6" t="s">
+      <c r="B12" s="8" t="n">
+        <v>0</v>
+      </c>
+      <c r="C12" s="8" t="n">
+        <v>0</v>
+      </c>
+      <c r="D12" s="8" t="n">
+        <v>0</v>
+      </c>
+      <c r="E12" s="8" t="n">
+        <v>0</v>
+      </c>
+      <c r="F12" s="8" t="n">
+        <v>0</v>
+      </c>
+      <c r="G12" s="8" t="n">
+        <v>0</v>
+      </c>
+      <c r="H12" s="8" t="n">
+        <v>0</v>
+      </c>
+      <c r="I12" s="8" t="n">
+        <v>0</v>
+      </c>
+      <c r="J12" s="8" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="13" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A13" s="7" t="s">
         <v>196</v>
       </c>
-      <c r="B13" s="6" t="n">
-        <v>0</v>
-      </c>
-      <c r="C13" s="6" t="n">
-        <v>0</v>
-      </c>
-      <c r="D13" s="6" t="n">
-        <v>0</v>
-      </c>
-      <c r="E13" s="6" t="n">
-        <v>0</v>
-      </c>
-      <c r="F13" s="6" t="n">
-        <v>0</v>
-      </c>
-      <c r="G13" s="6" t="n">
-        <v>0</v>
-      </c>
-      <c r="H13" s="6" t="n">
-        <v>0</v>
-      </c>
-      <c r="I13" s="6" t="n">
-        <v>0</v>
-      </c>
-      <c r="J13" s="6" t="n">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="14" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A14" s="7" t="s">
+      <c r="B13" s="7" t="n">
+        <v>0</v>
+      </c>
+      <c r="C13" s="7" t="n">
+        <v>0</v>
+      </c>
+      <c r="D13" s="7" t="n">
+        <v>0</v>
+      </c>
+      <c r="E13" s="7" t="n">
+        <v>0</v>
+      </c>
+      <c r="F13" s="7" t="n">
+        <v>0</v>
+      </c>
+      <c r="G13" s="7" t="n">
+        <v>0</v>
+      </c>
+      <c r="H13" s="7" t="n">
+        <v>0</v>
+      </c>
+      <c r="I13" s="7" t="n">
+        <v>0</v>
+      </c>
+      <c r="J13" s="7" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="14" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A14" s="8" t="s">
         <v>197</v>
       </c>
-      <c r="B14" s="7" t="n">
-        <v>0</v>
-      </c>
-      <c r="C14" s="7" t="n">
-        <v>0</v>
-      </c>
-      <c r="D14" s="7" t="n">
-        <v>0</v>
-      </c>
-      <c r="E14" s="7" t="n">
-        <v>0</v>
-      </c>
-      <c r="F14" s="7" t="n">
-        <v>0</v>
-      </c>
-      <c r="G14" s="7" t="n">
-        <v>0</v>
-      </c>
-      <c r="H14" s="7" t="n">
-        <v>0</v>
-      </c>
-      <c r="I14" s="7" t="n">
-        <v>0</v>
-      </c>
-      <c r="J14" s="7" t="n">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="15" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A15" s="8" t="s">
+      <c r="B14" s="8" t="n">
+        <v>0</v>
+      </c>
+      <c r="C14" s="8" t="n">
+        <v>0</v>
+      </c>
+      <c r="D14" s="8" t="n">
+        <v>0</v>
+      </c>
+      <c r="E14" s="8" t="n">
+        <v>0</v>
+      </c>
+      <c r="F14" s="8" t="n">
+        <v>0</v>
+      </c>
+      <c r="G14" s="8" t="n">
+        <v>0</v>
+      </c>
+      <c r="H14" s="8" t="n">
+        <v>0</v>
+      </c>
+      <c r="I14" s="8" t="n">
+        <v>0</v>
+      </c>
+      <c r="J14" s="8" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="15" customFormat="false" ht="23.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A15" s="9" t="s">
         <v>198</v>
       </c>
-      <c r="B15" s="8" t="n">
+      <c r="B15" s="9" t="n">
         <f aca="false">SUM(B3:B5)</f>
         <v>426500</v>
       </c>
-      <c r="C15" s="8" t="n">
+      <c r="C15" s="9" t="n">
         <f aca="false">AVERAGE(C3:C5)</f>
         <v>93.1666666666667</v>
       </c>
-      <c r="D15" s="8" t="n">
+      <c r="D15" s="9" t="n">
         <f aca="false">AVERAGE(D3:D5)</f>
         <v>88.3666666666667</v>
       </c>
-      <c r="E15" s="8" t="n">
+      <c r="E15" s="9" t="n">
         <f aca="false">AVERAGE(E3:E5)</f>
         <v>1.93333333333333</v>
       </c>
-      <c r="F15" s="8" t="n">
+      <c r="F15" s="9" t="n">
         <f aca="false">AVERAGE(F3:F5)</f>
         <v>1.73333333333333</v>
       </c>
-      <c r="G15" s="8" t="n">
+      <c r="G15" s="9" t="n">
         <f aca="false">AVERAGE(G3:G5)</f>
         <v>49.5666666666667</v>
       </c>
-      <c r="H15" s="8" t="n">
+      <c r="H15" s="9" t="n">
         <f aca="false">SUM(H3:H5)</f>
         <v>996</v>
       </c>
-      <c r="I15" s="8" t="n">
+      <c r="I15" s="9" t="n">
         <f aca="false">SUM(I3:I5)</f>
         <v>104</v>
       </c>
-      <c r="J15" s="8" t="n">
+      <c r="J15" s="9" t="n">
         <f aca="false">SUM(J3:J5)</f>
         <v>10</v>
       </c>
@@ -2954,443 +2958,443 @@
   <dimension ref="A1:J14"/>
   <sheetFormatPr defaultColWidth="8.6796875" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="28"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="2" style="0" width="14"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="4" min="4" style="0" width="16"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="6" min="5" style="0" width="20"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="7" min="7" style="0" width="16"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="8" min="8" style="0" width="28"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="9" min="9" style="0" width="20"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="10" min="10" style="0" width="16"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="1" width="28"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="2" style="1" width="14"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="4" min="4" style="1" width="16"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="6" min="5" style="1" width="20"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="7" min="7" style="1" width="16"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="8" min="8" style="1" width="28"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="9" min="9" style="1" width="20"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="10" min="10" style="1" width="16"/>
   </cols>
   <sheetData>
     <row r="1" customFormat="false" ht="27.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A1" s="1" t="s">
+      <c r="A1" s="2" t="s">
         <v>199</v>
       </c>
-      <c r="B1" s="1"/>
-      <c r="C1" s="1"/>
-      <c r="D1" s="1"/>
-      <c r="E1" s="1"/>
-      <c r="F1" s="1"/>
-      <c r="G1" s="1"/>
-      <c r="H1" s="1"/>
-      <c r="I1" s="1"/>
-      <c r="J1" s="1"/>
+      <c r="B1" s="2"/>
+      <c r="C1" s="2"/>
+      <c r="D1" s="2"/>
+      <c r="E1" s="2"/>
+      <c r="F1" s="2"/>
+      <c r="G1" s="2"/>
+      <c r="H1" s="2"/>
+      <c r="I1" s="2"/>
+      <c r="J1" s="2"/>
     </row>
     <row r="2" customFormat="false" ht="36" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A2" s="2" t="s">
+      <c r="A2" s="3" t="s">
         <v>27</v>
       </c>
-      <c r="B2" s="2" t="s">
+      <c r="B2" s="3" t="s">
         <v>200</v>
       </c>
-      <c r="C2" s="2" t="s">
+      <c r="C2" s="3" t="s">
         <v>201</v>
       </c>
-      <c r="D2" s="2" t="s">
+      <c r="D2" s="3" t="s">
         <v>202</v>
       </c>
-      <c r="E2" s="2" t="s">
+      <c r="E2" s="3" t="s">
         <v>203</v>
       </c>
-      <c r="F2" s="2" t="s">
+      <c r="F2" s="3" t="s">
         <v>204</v>
       </c>
-      <c r="G2" s="2" t="s">
+      <c r="G2" s="3" t="s">
         <v>205</v>
       </c>
-      <c r="H2" s="2" t="s">
+      <c r="H2" s="3" t="s">
         <v>206</v>
       </c>
-      <c r="I2" s="2" t="s">
+      <c r="I2" s="3" t="s">
         <v>207</v>
       </c>
-      <c r="J2" s="2" t="s">
+      <c r="J2" s="3" t="s">
         <v>208</v>
       </c>
     </row>
-    <row r="3" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A3" s="6" t="s">
+    <row r="3" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A3" s="7" t="s">
         <v>131</v>
       </c>
-      <c r="B3" s="6" t="n">
+      <c r="B3" s="7" t="n">
         <v>14</v>
       </c>
-      <c r="C3" s="6" t="n">
+      <c r="C3" s="7" t="n">
         <v>9</v>
       </c>
-      <c r="D3" s="6" t="n">
+      <c r="D3" s="7" t="n">
         <v>5</v>
       </c>
-      <c r="E3" s="6" t="n">
+      <c r="E3" s="7" t="n">
         <v>4.2</v>
       </c>
-      <c r="F3" s="6" t="n">
+      <c r="F3" s="7" t="n">
         <v>2</v>
       </c>
-      <c r="G3" s="6" t="n">
+      <c r="G3" s="7" t="n">
         <v>18</v>
       </c>
-      <c r="H3" s="6" t="s">
+      <c r="H3" s="7" t="s">
         <v>209</v>
       </c>
-      <c r="I3" s="6" t="s">
+      <c r="I3" s="7" t="s">
         <v>43</v>
       </c>
-      <c r="J3" s="6" t="n">
+      <c r="J3" s="7" t="n">
         <v>62</v>
       </c>
     </row>
-    <row r="4" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A4" s="7" t="s">
+    <row r="4" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A4" s="8" t="s">
         <v>123</v>
       </c>
-      <c r="B4" s="7" t="n">
+      <c r="B4" s="8" t="n">
         <v>18</v>
       </c>
-      <c r="C4" s="7" t="n">
+      <c r="C4" s="8" t="n">
         <v>7</v>
       </c>
-      <c r="D4" s="7" t="n">
+      <c r="D4" s="8" t="n">
         <v>11</v>
       </c>
-      <c r="E4" s="7" t="n">
+      <c r="E4" s="8" t="n">
         <v>6.8</v>
       </c>
-      <c r="F4" s="7" t="n">
+      <c r="F4" s="8" t="n">
         <v>4</v>
       </c>
-      <c r="G4" s="7" t="n">
+      <c r="G4" s="8" t="n">
         <v>12</v>
       </c>
-      <c r="H4" s="7" t="s">
+      <c r="H4" s="8" t="s">
         <v>210</v>
       </c>
-      <c r="I4" s="7" t="s">
+      <c r="I4" s="8" t="s">
         <v>66</v>
       </c>
-      <c r="J4" s="7" t="n">
+      <c r="J4" s="8" t="n">
         <v>71</v>
       </c>
     </row>
-    <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A5" s="6" t="s">
+    <row r="5" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A5" s="7" t="s">
         <v>138</v>
       </c>
-      <c r="B5" s="6" t="n">
+      <c r="B5" s="7" t="n">
         <v>12</v>
       </c>
-      <c r="C5" s="6" t="n">
+      <c r="C5" s="7" t="n">
         <v>5</v>
       </c>
-      <c r="D5" s="6" t="n">
+      <c r="D5" s="7" t="n">
         <v>7</v>
       </c>
-      <c r="E5" s="6" t="n">
+      <c r="E5" s="7" t="n">
         <v>1.4</v>
       </c>
-      <c r="F5" s="6" t="n">
+      <c r="F5" s="7" t="n">
         <v>1</v>
       </c>
-      <c r="G5" s="6" t="n">
+      <c r="G5" s="7" t="n">
         <v>8</v>
       </c>
-      <c r="H5" s="6" t="s">
+      <c r="H5" s="7" t="s">
         <v>211</v>
       </c>
-      <c r="I5" s="6" t="s">
+      <c r="I5" s="7" t="s">
         <v>43</v>
       </c>
-      <c r="J5" s="6" t="n">
+      <c r="J5" s="7" t="n">
         <v>76</v>
       </c>
     </row>
-    <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A6" s="7" t="s">
+    <row r="6" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A6" s="8" t="s">
         <v>212</v>
       </c>
-      <c r="B6" s="7" t="n">
+      <c r="B6" s="8" t="n">
         <v>10</v>
       </c>
-      <c r="C6" s="7" t="n">
+      <c r="C6" s="8" t="n">
         <v>8</v>
       </c>
-      <c r="D6" s="7" t="n">
+      <c r="D6" s="8" t="n">
         <v>2</v>
       </c>
-      <c r="E6" s="7" t="n">
+      <c r="E6" s="8" t="n">
         <v>48</v>
       </c>
-      <c r="F6" s="7" t="n">
+      <c r="F6" s="8" t="n">
         <v>24</v>
       </c>
-      <c r="G6" s="7" t="n">
+      <c r="G6" s="8" t="n">
         <v>22</v>
       </c>
-      <c r="H6" s="7" t="s">
+      <c r="H6" s="8" t="s">
         <v>213</v>
       </c>
-      <c r="I6" s="7" t="s">
+      <c r="I6" s="8" t="s">
         <v>43</v>
       </c>
-      <c r="J6" s="7" t="n">
+      <c r="J6" s="8" t="n">
         <v>41</v>
       </c>
     </row>
-    <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A7" s="6" t="s">
+    <row r="7" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A7" s="7" t="s">
         <v>214</v>
       </c>
-      <c r="B7" s="6" t="n">
+      <c r="B7" s="7" t="n">
         <v>8</v>
       </c>
-      <c r="C7" s="6" t="n">
+      <c r="C7" s="7" t="n">
         <v>6</v>
       </c>
-      <c r="D7" s="6" t="n">
+      <c r="D7" s="7" t="n">
         <v>2</v>
       </c>
-      <c r="E7" s="6" t="n">
+      <c r="E7" s="7" t="n">
         <v>9.2</v>
       </c>
-      <c r="F7" s="6" t="n">
+      <c r="F7" s="7" t="n">
         <v>4</v>
       </c>
-      <c r="G7" s="6" t="n">
+      <c r="G7" s="7" t="n">
         <v>15</v>
       </c>
-      <c r="H7" s="6" t="s">
+      <c r="H7" s="7" t="s">
         <v>215</v>
       </c>
-      <c r="I7" s="6" t="s">
+      <c r="I7" s="7" t="s">
         <v>66</v>
       </c>
-      <c r="J7" s="6" t="n">
+      <c r="J7" s="7" t="n">
         <v>55</v>
       </c>
     </row>
-    <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A8" s="7" t="s">
+    <row r="8" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A8" s="8" t="s">
         <v>152</v>
       </c>
-      <c r="B8" s="7" t="n">
+      <c r="B8" s="8" t="n">
         <v>11</v>
       </c>
-      <c r="C8" s="7" t="n">
+      <c r="C8" s="8" t="n">
         <v>9</v>
       </c>
-      <c r="D8" s="7" t="n">
+      <c r="D8" s="8" t="n">
         <v>2</v>
       </c>
-      <c r="E8" s="7" t="n">
+      <c r="E8" s="8" t="n">
         <v>72</v>
       </c>
-      <c r="F8" s="7" t="n">
+      <c r="F8" s="8" t="n">
         <v>48</v>
       </c>
-      <c r="G8" s="7" t="n">
+      <c r="G8" s="8" t="n">
         <v>31</v>
       </c>
-      <c r="H8" s="7" t="s">
+      <c r="H8" s="8" t="s">
         <v>216</v>
       </c>
-      <c r="I8" s="7" t="s">
+      <c r="I8" s="8" t="s">
         <v>43</v>
       </c>
-      <c r="J8" s="7" t="n">
+      <c r="J8" s="8" t="n">
         <v>38</v>
       </c>
     </row>
-    <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A9" s="6" t="s">
+    <row r="9" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A9" s="7" t="s">
         <v>162</v>
       </c>
-      <c r="B9" s="6" t="n">
+      <c r="B9" s="7" t="n">
         <v>9</v>
       </c>
-      <c r="C9" s="6" t="n">
+      <c r="C9" s="7" t="n">
         <v>8</v>
       </c>
-      <c r="D9" s="6" t="n">
+      <c r="D9" s="7" t="n">
         <v>1</v>
       </c>
-      <c r="E9" s="6" t="n">
+      <c r="E9" s="7" t="n">
         <v>2.8</v>
       </c>
-      <c r="F9" s="6" t="n">
+      <c r="F9" s="7" t="n">
         <v>1.5</v>
       </c>
-      <c r="G9" s="6" t="n">
+      <c r="G9" s="7" t="n">
         <v>6</v>
       </c>
-      <c r="H9" s="6" t="s">
+      <c r="H9" s="7" t="s">
         <v>217</v>
       </c>
-      <c r="I9" s="6" t="s">
+      <c r="I9" s="7" t="s">
         <v>92</v>
       </c>
-      <c r="J9" s="6" t="n">
+      <c r="J9" s="7" t="n">
         <v>52</v>
       </c>
     </row>
-    <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A10" s="7" t="s">
+    <row r="10" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A10" s="8" t="s">
         <v>218</v>
       </c>
-      <c r="B10" s="7" t="n">
+      <c r="B10" s="8" t="n">
         <v>16</v>
       </c>
-      <c r="C10" s="7" t="n">
+      <c r="C10" s="8" t="n">
         <v>14</v>
       </c>
-      <c r="D10" s="7" t="n">
+      <c r="D10" s="8" t="n">
         <v>2</v>
       </c>
-      <c r="E10" s="7" t="n">
+      <c r="E10" s="8" t="n">
         <v>120</v>
       </c>
-      <c r="F10" s="7" t="n">
+      <c r="F10" s="8" t="n">
         <v>48</v>
       </c>
-      <c r="G10" s="7" t="n">
+      <c r="G10" s="8" t="n">
         <v>25</v>
       </c>
-      <c r="H10" s="7" t="s">
+      <c r="H10" s="8" t="s">
         <v>219</v>
       </c>
-      <c r="I10" s="7" t="s">
+      <c r="I10" s="8" t="s">
         <v>43</v>
       </c>
-      <c r="J10" s="7" t="n">
+      <c r="J10" s="8" t="n">
         <v>30</v>
       </c>
     </row>
-    <row r="11" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A11" s="6" t="s">
+    <row r="11" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A11" s="7" t="s">
         <v>148</v>
       </c>
-      <c r="B11" s="6" t="n">
+      <c r="B11" s="7" t="n">
         <v>7</v>
       </c>
-      <c r="C11" s="6" t="n">
+      <c r="C11" s="7" t="n">
         <v>3</v>
       </c>
-      <c r="D11" s="6" t="n">
+      <c r="D11" s="7" t="n">
         <v>4</v>
       </c>
-      <c r="E11" s="6" t="n">
+      <c r="E11" s="7" t="n">
         <v>36</v>
       </c>
-      <c r="F11" s="6" t="n">
+      <c r="F11" s="7" t="n">
         <v>24</v>
       </c>
-      <c r="G11" s="6" t="n">
+      <c r="G11" s="7" t="n">
         <v>10</v>
       </c>
-      <c r="H11" s="6" t="s">
+      <c r="H11" s="7" t="s">
         <v>220</v>
       </c>
-      <c r="I11" s="6" t="s">
+      <c r="I11" s="7" t="s">
         <v>66</v>
       </c>
-      <c r="J11" s="6" t="n">
+      <c r="J11" s="7" t="n">
         <v>64</v>
       </c>
     </row>
-    <row r="12" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A12" s="7" t="s">
+    <row r="12" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A12" s="8" t="s">
         <v>221</v>
       </c>
-      <c r="B12" s="7" t="n">
+      <c r="B12" s="8" t="n">
         <v>13</v>
       </c>
-      <c r="C12" s="7" t="n">
+      <c r="C12" s="8" t="n">
         <v>10</v>
       </c>
-      <c r="D12" s="7" t="n">
+      <c r="D12" s="8" t="n">
         <v>3</v>
       </c>
-      <c r="E12" s="7" t="n">
+      <c r="E12" s="8" t="n">
         <v>96</v>
       </c>
-      <c r="F12" s="7" t="n">
+      <c r="F12" s="8" t="n">
         <v>48</v>
       </c>
-      <c r="G12" s="7" t="n">
+      <c r="G12" s="8" t="n">
         <v>20</v>
       </c>
-      <c r="H12" s="7" t="s">
+      <c r="H12" s="8" t="s">
         <v>222</v>
       </c>
-      <c r="I12" s="7" t="s">
+      <c r="I12" s="8" t="s">
         <v>43</v>
       </c>
-      <c r="J12" s="7" t="n">
+      <c r="J12" s="8" t="n">
         <v>45</v>
       </c>
     </row>
-    <row r="13" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A13" s="6" t="s">
+    <row r="13" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A13" s="7" t="s">
         <v>143</v>
       </c>
-      <c r="B13" s="6" t="n">
+      <c r="B13" s="7" t="n">
         <v>8</v>
       </c>
-      <c r="C13" s="6" t="n">
+      <c r="C13" s="7" t="n">
         <v>6</v>
       </c>
-      <c r="D13" s="6" t="n">
+      <c r="D13" s="7" t="n">
         <v>2</v>
       </c>
-      <c r="E13" s="6" t="n">
+      <c r="E13" s="7" t="n">
         <v>18</v>
       </c>
-      <c r="F13" s="6" t="n">
+      <c r="F13" s="7" t="n">
         <v>8</v>
       </c>
-      <c r="G13" s="6" t="n">
+      <c r="G13" s="7" t="n">
         <v>14</v>
       </c>
-      <c r="H13" s="6" t="s">
+      <c r="H13" s="7" t="s">
         <v>223</v>
       </c>
-      <c r="I13" s="6" t="s">
+      <c r="I13" s="7" t="s">
         <v>66</v>
       </c>
-      <c r="J13" s="6" t="n">
+      <c r="J13" s="7" t="n">
         <v>58</v>
       </c>
     </row>
-    <row r="14" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A14" s="7" t="s">
+    <row r="14" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A14" s="8" t="s">
         <v>94</v>
       </c>
-      <c r="B14" s="7" t="n">
+      <c r="B14" s="8" t="n">
         <v>6</v>
       </c>
-      <c r="C14" s="7" t="n">
+      <c r="C14" s="8" t="n">
         <v>1</v>
       </c>
-      <c r="D14" s="7" t="n">
+      <c r="D14" s="8" t="n">
         <v>5</v>
       </c>
-      <c r="E14" s="7" t="n">
+      <c r="E14" s="8" t="n">
         <v>0.8</v>
       </c>
-      <c r="F14" s="7" t="n">
+      <c r="F14" s="8" t="n">
         <v>0.5</v>
       </c>
-      <c r="G14" s="7" t="n">
+      <c r="G14" s="8" t="n">
         <v>3</v>
       </c>
-      <c r="H14" s="7" t="s">
+      <c r="H14" s="8" t="s">
         <v>224</v>
       </c>
-      <c r="I14" s="7" t="s">
+      <c r="I14" s="8" t="s">
         <v>92</v>
       </c>
-      <c r="J14" s="7" t="n">
+      <c r="J14" s="8" t="n">
         <v>85</v>
       </c>
     </row>
@@ -3416,380 +3420,380 @@
   <dimension ref="A1:J12"/>
   <sheetFormatPr defaultColWidth="8.6796875" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="12"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="0" width="14"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="3" style="0" width="20"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="4" min="4" style="0" width="44"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="5" min="5" style="0" width="26"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="6" min="6" style="0" width="22"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="7" min="7" style="0" width="52"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="8" min="8" style="0" width="36"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="10" min="9" style="0" width="14"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="1" width="12"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="1" width="14"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="3" style="1" width="20"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="4" min="4" style="1" width="44"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="5" min="5" style="1" width="26"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="6" min="6" style="1" width="22"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="7" min="7" style="1" width="52"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="8" min="8" style="1" width="36"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="10" min="9" style="1" width="14"/>
   </cols>
   <sheetData>
     <row r="1" customFormat="false" ht="27.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A1" s="1" t="s">
+      <c r="A1" s="2" t="s">
         <v>225</v>
       </c>
-      <c r="B1" s="1"/>
-      <c r="C1" s="1"/>
-      <c r="D1" s="1"/>
-      <c r="E1" s="1"/>
-      <c r="F1" s="1"/>
-      <c r="G1" s="1"/>
-      <c r="H1" s="1"/>
-      <c r="I1" s="1"/>
-      <c r="J1" s="1"/>
+      <c r="B1" s="2"/>
+      <c r="C1" s="2"/>
+      <c r="D1" s="2"/>
+      <c r="E1" s="2"/>
+      <c r="F1" s="2"/>
+      <c r="G1" s="2"/>
+      <c r="H1" s="2"/>
+      <c r="I1" s="2"/>
+      <c r="J1" s="2"/>
     </row>
     <row r="2" customFormat="false" ht="36" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A2" s="2" t="s">
+      <c r="A2" s="3" t="s">
         <v>226</v>
       </c>
-      <c r="B2" s="2" t="s">
+      <c r="B2" s="3" t="s">
         <v>112</v>
       </c>
-      <c r="C2" s="2" t="s">
+      <c r="C2" s="3" t="s">
         <v>227</v>
       </c>
-      <c r="D2" s="2" t="s">
+      <c r="D2" s="3" t="s">
         <v>228</v>
       </c>
-      <c r="E2" s="2" t="s">
+      <c r="E2" s="3" t="s">
         <v>229</v>
       </c>
-      <c r="F2" s="2" t="s">
+      <c r="F2" s="3" t="s">
         <v>230</v>
       </c>
-      <c r="G2" s="2" t="s">
+      <c r="G2" s="3" t="s">
         <v>231</v>
       </c>
-      <c r="H2" s="2" t="s">
+      <c r="H2" s="3" t="s">
         <v>232</v>
       </c>
-      <c r="I2" s="2" t="s">
+      <c r="I2" s="3" t="s">
         <v>233</v>
       </c>
-      <c r="J2" s="2" t="s">
+      <c r="J2" s="3" t="s">
         <v>33</v>
       </c>
     </row>
-    <row r="3" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A3" s="6" t="s">
+    <row r="3" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A3" s="7" t="s">
         <v>234</v>
       </c>
-      <c r="B3" s="6" t="s">
+      <c r="B3" s="7" t="s">
         <v>235</v>
       </c>
-      <c r="C3" s="6" t="s">
+      <c r="C3" s="7" t="s">
         <v>236</v>
       </c>
-      <c r="D3" s="6" t="s">
+      <c r="D3" s="7" t="s">
         <v>237</v>
       </c>
-      <c r="E3" s="6" t="s">
+      <c r="E3" s="7" t="s">
         <v>238</v>
       </c>
-      <c r="F3" s="6" t="s">
+      <c r="F3" s="7" t="s">
         <v>239</v>
       </c>
-      <c r="G3" s="6" t="s">
+      <c r="G3" s="7" t="s">
         <v>240</v>
       </c>
-      <c r="H3" s="6" t="s">
+      <c r="H3" s="7" t="s">
         <v>241</v>
       </c>
-      <c r="I3" s="6" t="s">
+      <c r="I3" s="7" t="s">
         <v>122</v>
       </c>
-      <c r="J3" s="6" t="s">
+      <c r="J3" s="7" t="s">
         <v>242</v>
       </c>
     </row>
-    <row r="4" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A4" s="7" t="s">
+    <row r="4" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A4" s="8" t="s">
         <v>243</v>
       </c>
-      <c r="B4" s="7" t="s">
+      <c r="B4" s="8" t="s">
         <v>122</v>
       </c>
-      <c r="C4" s="7" t="s">
+      <c r="C4" s="8" t="s">
         <v>244</v>
       </c>
-      <c r="D4" s="7" t="s">
+      <c r="D4" s="8" t="s">
         <v>245</v>
       </c>
-      <c r="E4" s="7" t="s">
+      <c r="E4" s="8" t="s">
         <v>246</v>
       </c>
-      <c r="F4" s="7" t="s">
+      <c r="F4" s="8" t="s">
         <v>247</v>
       </c>
-      <c r="G4" s="7" t="s">
+      <c r="G4" s="8" t="s">
         <v>248</v>
       </c>
-      <c r="H4" s="7" t="s">
+      <c r="H4" s="8" t="s">
         <v>249</v>
       </c>
-      <c r="I4" s="7" t="s">
+      <c r="I4" s="8" t="s">
         <v>250</v>
       </c>
-      <c r="J4" s="7" t="s">
+      <c r="J4" s="8" t="s">
         <v>251</v>
       </c>
     </row>
-    <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A5" s="6" t="s">
+    <row r="5" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A5" s="7" t="s">
         <v>252</v>
       </c>
-      <c r="B5" s="6" t="s">
+      <c r="B5" s="7" t="s">
         <v>130</v>
       </c>
-      <c r="C5" s="6" t="s">
+      <c r="C5" s="7" t="s">
         <v>253</v>
       </c>
-      <c r="D5" s="6" t="s">
+      <c r="D5" s="7" t="s">
         <v>254</v>
       </c>
-      <c r="E5" s="6" t="s">
+      <c r="E5" s="7" t="s">
         <v>255</v>
       </c>
-      <c r="F5" s="6" t="s">
+      <c r="F5" s="7" t="s">
         <v>98</v>
       </c>
-      <c r="G5" s="6" t="s">
+      <c r="G5" s="7" t="s">
         <v>256</v>
       </c>
-      <c r="H5" s="6" t="s">
+      <c r="H5" s="7" t="s">
         <v>257</v>
       </c>
-      <c r="I5" s="6" t="s">
+      <c r="I5" s="7" t="s">
         <v>258</v>
       </c>
-      <c r="J5" s="6" t="s">
+      <c r="J5" s="7" t="s">
         <v>259</v>
       </c>
     </row>
-    <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A6" s="7" t="s">
+    <row r="6" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A6" s="8" t="s">
         <v>260</v>
       </c>
-      <c r="B6" s="7" t="s">
+      <c r="B6" s="8" t="s">
         <v>261</v>
       </c>
-      <c r="C6" s="7" t="s">
+      <c r="C6" s="8" t="s">
         <v>262</v>
       </c>
-      <c r="D6" s="7" t="s">
+      <c r="D6" s="8" t="s">
         <v>263</v>
       </c>
-      <c r="E6" s="7" t="s">
+      <c r="E6" s="8" t="s">
         <v>264</v>
       </c>
-      <c r="F6" s="7" t="s">
+      <c r="F6" s="8" t="s">
         <v>265</v>
       </c>
-      <c r="G6" s="7" t="s">
+      <c r="G6" s="8" t="s">
         <v>266</v>
       </c>
-      <c r="H6" s="7" t="s">
+      <c r="H6" s="8" t="s">
         <v>267</v>
       </c>
-      <c r="I6" s="7" t="s">
+      <c r="I6" s="8" t="s">
         <v>268</v>
       </c>
-      <c r="J6" s="7" t="s">
+      <c r="J6" s="8" t="s">
         <v>242</v>
       </c>
     </row>
-    <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A7" s="6" t="s">
+    <row r="7" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A7" s="7" t="s">
         <v>269</v>
       </c>
-      <c r="B7" s="6" t="s">
+      <c r="B7" s="7" t="s">
         <v>147</v>
       </c>
-      <c r="C7" s="6" t="s">
+      <c r="C7" s="7" t="s">
         <v>270</v>
       </c>
-      <c r="D7" s="6" t="s">
+      <c r="D7" s="7" t="s">
         <v>271</v>
       </c>
-      <c r="E7" s="6" t="s">
+      <c r="E7" s="7" t="s">
         <v>272</v>
       </c>
-      <c r="F7" s="6" t="s">
+      <c r="F7" s="7" t="s">
         <v>273</v>
       </c>
-      <c r="G7" s="6" t="s">
+      <c r="G7" s="7" t="s">
         <v>274</v>
       </c>
-      <c r="H7" s="6" t="s">
+      <c r="H7" s="7" t="s">
         <v>275</v>
       </c>
-      <c r="I7" s="6" t="s">
+      <c r="I7" s="7" t="s">
         <v>276</v>
       </c>
-      <c r="J7" s="6" t="s">
+      <c r="J7" s="7" t="s">
         <v>180</v>
       </c>
     </row>
-    <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A8" s="7" t="s">
+    <row r="8" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A8" s="8" t="s">
         <v>277</v>
       </c>
-      <c r="B8" s="7" t="s">
+      <c r="B8" s="8" t="s">
         <v>151</v>
       </c>
-      <c r="C8" s="7" t="s">
+      <c r="C8" s="8" t="s">
         <v>278</v>
       </c>
-      <c r="D8" s="7" t="s">
+      <c r="D8" s="8" t="s">
         <v>279</v>
       </c>
-      <c r="E8" s="7" t="s">
+      <c r="E8" s="8" t="s">
         <v>280</v>
       </c>
-      <c r="F8" s="7" t="s">
+      <c r="F8" s="8" t="s">
         <v>281</v>
       </c>
-      <c r="G8" s="7" t="s">
+      <c r="G8" s="8" t="s">
         <v>282</v>
       </c>
-      <c r="H8" s="7" t="s">
+      <c r="H8" s="8" t="s">
         <v>283</v>
       </c>
-      <c r="I8" s="7" t="s">
+      <c r="I8" s="8" t="s">
         <v>284</v>
       </c>
-      <c r="J8" s="7" t="s">
+      <c r="J8" s="8" t="s">
         <v>242</v>
       </c>
     </row>
-    <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A9" s="6" t="s">
+    <row r="9" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A9" s="7" t="s">
         <v>285</v>
       </c>
-      <c r="B9" s="6" t="s">
+      <c r="B9" s="7" t="s">
         <v>286</v>
       </c>
-      <c r="C9" s="6" t="s">
+      <c r="C9" s="7" t="s">
         <v>262</v>
       </c>
-      <c r="D9" s="6" t="s">
+      <c r="D9" s="7" t="s">
         <v>287</v>
       </c>
-      <c r="E9" s="6" t="s">
+      <c r="E9" s="7" t="s">
         <v>264</v>
       </c>
-      <c r="F9" s="6" t="s">
+      <c r="F9" s="7" t="s">
         <v>265</v>
       </c>
-      <c r="G9" s="6" t="s">
+      <c r="G9" s="7" t="s">
         <v>288</v>
       </c>
-      <c r="H9" s="6" t="s">
+      <c r="H9" s="7" t="s">
         <v>289</v>
       </c>
-      <c r="I9" s="6" t="s">
+      <c r="I9" s="7" t="s">
         <v>173</v>
       </c>
-      <c r="J9" s="6" t="s">
+      <c r="J9" s="7" t="s">
         <v>290</v>
       </c>
     </row>
-    <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A10" s="7" t="s">
+    <row r="10" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A10" s="8" t="s">
         <v>291</v>
       </c>
-      <c r="B10" s="7" t="s">
+      <c r="B10" s="8" t="s">
         <v>170</v>
       </c>
-      <c r="C10" s="7" t="s">
+      <c r="C10" s="8" t="s">
         <v>244</v>
       </c>
-      <c r="D10" s="7" t="s">
+      <c r="D10" s="8" t="s">
         <v>292</v>
       </c>
-      <c r="E10" s="7" t="s">
+      <c r="E10" s="8" t="s">
         <v>293</v>
       </c>
-      <c r="F10" s="7" t="s">
+      <c r="F10" s="8" t="s">
         <v>247</v>
       </c>
-      <c r="G10" s="7" t="s">
+      <c r="G10" s="8" t="s">
         <v>294</v>
       </c>
-      <c r="H10" s="7" t="s">
+      <c r="H10" s="8" t="s">
         <v>295</v>
       </c>
-      <c r="I10" s="7" t="s">
+      <c r="I10" s="8" t="s">
         <v>296</v>
       </c>
-      <c r="J10" s="7" t="s">
+      <c r="J10" s="8" t="s">
         <v>242</v>
       </c>
     </row>
-    <row r="11" customFormat="false" ht="22.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A11" s="6" t="s">
+    <row r="11" customFormat="false" ht="21.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A11" s="7" t="s">
         <v>297</v>
       </c>
-      <c r="B11" s="6" t="s">
+      <c r="B11" s="7" t="s">
         <v>173</v>
       </c>
-      <c r="C11" s="6" t="s">
+      <c r="C11" s="7" t="s">
         <v>270</v>
       </c>
-      <c r="D11" s="6" t="s">
+      <c r="D11" s="7" t="s">
         <v>298</v>
       </c>
-      <c r="E11" s="6" t="s">
+      <c r="E11" s="7" t="s">
         <v>299</v>
       </c>
-      <c r="F11" s="6" t="s">
+      <c r="F11" s="7" t="s">
         <v>300</v>
       </c>
-      <c r="G11" s="6" t="s">
+      <c r="G11" s="7" t="s">
         <v>301</v>
       </c>
-      <c r="H11" s="6" t="s">
+      <c r="H11" s="7" t="s">
         <v>302</v>
       </c>
-      <c r="I11" s="6" t="s">
+      <c r="I11" s="7" t="s">
         <v>303</v>
       </c>
-      <c r="J11" s="6" t="s">
+      <c r="J11" s="7" t="s">
         <v>101</v>
       </c>
     </row>
-    <row r="12" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A12" s="7" t="s">
+    <row r="12" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A12" s="8" t="s">
         <v>304</v>
       </c>
-      <c r="B12" s="7" t="s">
+      <c r="B12" s="8" t="s">
         <v>173</v>
       </c>
-      <c r="C12" s="7" t="s">
+      <c r="C12" s="8" t="s">
         <v>305</v>
       </c>
-      <c r="D12" s="7" t="s">
+      <c r="D12" s="8" t="s">
         <v>306</v>
       </c>
-      <c r="E12" s="7" t="s">
+      <c r="E12" s="8" t="s">
         <v>307</v>
       </c>
-      <c r="F12" s="7" t="s">
+      <c r="F12" s="8" t="s">
         <v>239</v>
       </c>
-      <c r="G12" s="7" t="s">
+      <c r="G12" s="8" t="s">
         <v>308</v>
       </c>
-      <c r="H12" s="7" t="s">
+      <c r="H12" s="8" t="s">
         <v>309</v>
       </c>
-      <c r="I12" s="7" t="s">
+      <c r="I12" s="8" t="s">
         <v>303</v>
       </c>
-      <c r="J12" s="7" t="s">
+      <c r="J12" s="8" t="s">
         <v>259</v>
       </c>
     </row>

</xml_diff>